<commit_message>
Corrected links for Film and Film Craft
</commit_message>
<xml_diff>
--- a/Brain_Cannesdy_Brand_Experience_2025.xlsx
+++ b/Brain_Cannesdy_Brand_Experience_2025.xlsx
@@ -9997,7 +9997,7 @@
       </c>
       <c r="J4" s="33" t="inlineStr">
         <is>
-          <t>aoOfn_W8PWg</t>
+          <t>vimeo:974346956</t>
         </is>
       </c>
       <c r="L4" s="33" t="inlineStr">
@@ -31672,7 +31672,7 @@
       </c>
       <c r="J3" s="99" t="inlineStr">
         <is>
-          <t>-4o8bCc6-GM</t>
+          <t>vimeo:1094956645</t>
         </is>
       </c>
       <c r="L3" s="33" t="inlineStr">
@@ -31727,7 +31727,7 @@
       </c>
       <c r="J4" s="99" t="inlineStr">
         <is>
-          <t>LO4wamMlCKQ</t>
+          <t>vimeo:1068530073</t>
         </is>
       </c>
       <c r="K4" s="33" t="n"/>
@@ -32003,7 +32003,7 @@
       </c>
       <c r="J9" s="99" t="inlineStr">
         <is>
-          <t>DvaU3-VCk8I</t>
+          <t>vimeo:1081954251</t>
         </is>
       </c>
       <c r="L9" s="33" t="inlineStr">
@@ -32113,7 +32113,7 @@
       </c>
       <c r="J11" s="99" t="inlineStr">
         <is>
-          <t>cH8-sNMfrOM</t>
+          <t>vimeo:1158349533</t>
         </is>
       </c>
       <c r="L11" s="33" t="inlineStr">
@@ -32168,7 +32168,7 @@
       </c>
       <c r="J12" s="99" t="inlineStr">
         <is>
-          <t>jom8zBix-4c</t>
+          <t>vimeo:1006144786</t>
         </is>
       </c>
       <c r="L12" s="33" t="inlineStr">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="J13" s="99" t="inlineStr">
         <is>
-          <t>L-upphAEYGc</t>
+          <t>vimeo:1053855569</t>
         </is>
       </c>
       <c r="K13" s="33" t="n"/>
@@ -32279,7 +32279,7 @@
       </c>
       <c r="J14" s="99" t="inlineStr">
         <is>
-          <t>FFFmnfdBrm8</t>
+          <t>vimeo:1059963620</t>
         </is>
       </c>
       <c r="K14" s="33" t="n"/>
@@ -32335,7 +32335,7 @@
       </c>
       <c r="J15" s="99" t="inlineStr">
         <is>
-          <t>vimeo:1084058452</t>
+          <t>vimeo:1095860505</t>
         </is>
       </c>
       <c r="L15" s="33" t="inlineStr">
@@ -32390,7 +32390,7 @@
       </c>
       <c r="J16" s="99" t="inlineStr">
         <is>
-          <t>LXQtg237SKY</t>
+          <t>vimeo:1053465598</t>
         </is>
       </c>
       <c r="L16" s="33" t="inlineStr">
@@ -32445,7 +32445,7 @@
       </c>
       <c r="J17" s="99" t="inlineStr">
         <is>
-          <t>gGXMP0PpimM</t>
+          <t>vimeo:1026354274</t>
         </is>
       </c>
       <c r="K17" s="33" t="n"/>
@@ -32611,7 +32611,7 @@
       </c>
       <c r="J20" s="99" t="inlineStr">
         <is>
-          <t>9vpZNqaMVaQ</t>
+          <t>-saAXmItj_U</t>
         </is>
       </c>
       <c r="L20" s="33" t="inlineStr">
@@ -32776,7 +32776,7 @@
       </c>
       <c r="J23" s="99" t="inlineStr">
         <is>
-          <t>4P6ltRZaCLU</t>
+          <t>vimeo:1152992898</t>
         </is>
       </c>
       <c r="L23" s="33" t="inlineStr">
@@ -32831,7 +32831,7 @@
       </c>
       <c r="J24" s="99" t="inlineStr">
         <is>
-          <t>LO4wamMlCKQ</t>
+          <t>vimeo:1067749538</t>
         </is>
       </c>
       <c r="L24" s="33" t="inlineStr">
@@ -32941,7 +32941,7 @@
       </c>
       <c r="J26" s="99" t="inlineStr">
         <is>
-          <t>udite96Jhl8</t>
+          <t>vimeo:1092244065</t>
         </is>
       </c>
       <c r="L26" s="33" t="inlineStr">
@@ -32996,7 +32996,7 @@
       </c>
       <c r="J27" s="99" t="inlineStr">
         <is>
-          <t>Bcpu-jqAL6w</t>
+          <t>vimeo:1055257520</t>
         </is>
       </c>
       <c r="K27" s="33" t="n"/>
@@ -33052,7 +33052,7 @@
       </c>
       <c r="J28" s="99" t="inlineStr">
         <is>
-          <t>mSPou5OfPyw</t>
+          <t>vimeo:997540972</t>
         </is>
       </c>
       <c r="L28" s="33" t="inlineStr">
@@ -33217,7 +33217,7 @@
       </c>
       <c r="J31" s="99" t="inlineStr">
         <is>
-          <t>_I-QedV87Nw</t>
+          <t>vimeo:1028285893</t>
         </is>
       </c>
       <c r="L31" s="33" t="inlineStr">
@@ -33272,7 +33272,7 @@
       </c>
       <c r="J32" s="99" t="inlineStr">
         <is>
-          <t>AbLLBcDM064</t>
+          <t>P-45kC6zwlE</t>
         </is>
       </c>
       <c r="L32" s="33" t="inlineStr">
@@ -33438,7 +33438,7 @@
       </c>
       <c r="J35" s="99" t="inlineStr">
         <is>
-          <t>uXaZyGTQNKw</t>
+          <t>vimeo:1090341135</t>
         </is>
       </c>
       <c r="L35" s="33" t="inlineStr">
@@ -33493,7 +33493,7 @@
       </c>
       <c r="J36" s="99" t="inlineStr">
         <is>
-          <t>OXK-4pQhM7o</t>
+          <t>vimeo:1099522427</t>
         </is>
       </c>
       <c r="L36" s="33" t="inlineStr">
@@ -33548,7 +33548,7 @@
       </c>
       <c r="J37" s="99" t="inlineStr">
         <is>
-          <t>s5iVbNCmAJg</t>
+          <t>vimeo:935890559</t>
         </is>
       </c>
       <c r="L37" s="33" t="inlineStr">
@@ -33824,7 +33824,7 @@
       </c>
       <c r="J42" s="99" t="inlineStr">
         <is>
-          <t>lP8LLIjCe6Q</t>
+          <t>vimeo:1124774457</t>
         </is>
       </c>
       <c r="L42" s="33" t="inlineStr">
@@ -33989,7 +33989,7 @@
       </c>
       <c r="J45" s="99" t="inlineStr">
         <is>
-          <t>BoVS5Yq_H18</t>
+          <t>u0c7pO99Ysw</t>
         </is>
       </c>
       <c r="L45" s="33" t="inlineStr">
@@ -34044,7 +34044,7 @@
       </c>
       <c r="J46" s="99" t="inlineStr">
         <is>
-          <t>aoOfn_W8PWg</t>
+          <t>vimeo:974346956</t>
         </is>
       </c>
       <c r="L46" s="33" t="inlineStr">
@@ -34099,7 +34099,7 @@
       </c>
       <c r="J47" s="99" t="inlineStr">
         <is>
-          <t>RBQ-IoHfimQ</t>
+          <t>vimeo:1017294125</t>
         </is>
       </c>
       <c r="L47" s="33" t="inlineStr">
@@ -34319,7 +34319,7 @@
       </c>
       <c r="J51" s="99" t="inlineStr">
         <is>
-          <t>L265a4WchmA</t>
+          <t>vimeo:951306460</t>
         </is>
       </c>
       <c r="L51" s="33" t="inlineStr">
@@ -49605,7 +49605,7 @@
       </c>
       <c r="J6" s="33" t="inlineStr">
         <is>
-          <t>LO4wamMlCKQ</t>
+          <t>vimeo:1068530073</t>
         </is>
       </c>
       <c r="L6" s="33" t="inlineStr">
@@ -49715,7 +49715,7 @@
       </c>
       <c r="J8" s="33" t="inlineStr">
         <is>
-          <t>LXQtg237SKY</t>
+          <t>vimeo:1053465598</t>
         </is>
       </c>
       <c r="L8" s="33" t="inlineStr">
@@ -49885,7 +49885,7 @@
       </c>
       <c r="J11" s="33" t="inlineStr">
         <is>
-          <t>IQovoot_ZUM</t>
+          <t>_n5ZDERgrdc</t>
         </is>
       </c>
       <c r="L11" s="33" t="inlineStr">
@@ -50040,7 +50040,7 @@
       </c>
       <c r="J14" s="33" t="inlineStr">
         <is>
-          <t>FFFmnfdBrm8</t>
+          <t>vimeo:1010739490</t>
         </is>
       </c>
       <c r="L14" s="33" t="inlineStr">
@@ -50095,7 +50095,7 @@
       </c>
       <c r="J15" s="33" t="inlineStr">
         <is>
-          <t>LXQtg237SKY</t>
+          <t>vimeo:1053465598</t>
         </is>
       </c>
       <c r="L15" s="33" t="inlineStr">
@@ -50150,7 +50150,7 @@
       </c>
       <c r="J16" s="33" t="inlineStr">
         <is>
-          <t>jom8zBix-4c</t>
+          <t>vimeo:1006144786</t>
         </is>
       </c>
       <c r="K16" s="33" t="inlineStr">
@@ -50380,7 +50380,7 @@
       </c>
       <c r="J20" s="33" t="inlineStr">
         <is>
-          <t>hlqerWZSCpE</t>
+          <t>vimeo:1023704952</t>
         </is>
       </c>
       <c r="L20" s="33" t="inlineStr">
@@ -50435,7 +50435,7 @@
       </c>
       <c r="J21" s="33" t="inlineStr">
         <is>
-          <t>IQovoot_ZUM</t>
+          <t>_n5ZDERgrdc</t>
         </is>
       </c>
       <c r="L21" s="33" t="inlineStr">
@@ -50545,7 +50545,7 @@
       </c>
       <c r="J23" s="33" t="inlineStr">
         <is>
-          <t>Pb4SnxpJLyE</t>
+          <t>vimeo:958338280</t>
         </is>
       </c>
       <c r="L23" s="33" t="inlineStr">
@@ -50600,7 +50600,7 @@
       </c>
       <c r="J24" s="33" t="inlineStr">
         <is>
-          <t>jom8zBix-4c</t>
+          <t>vimeo:1006144786</t>
         </is>
       </c>
       <c r="K24" s="33" t="inlineStr">
@@ -50880,7 +50880,7 @@
       </c>
       <c r="J29" s="33" t="inlineStr">
         <is>
-          <t>LXQtg237SKY</t>
+          <t>vimeo:1053465598</t>
         </is>
       </c>
       <c r="L29" s="33" t="inlineStr">
@@ -50935,7 +50935,7 @@
       </c>
       <c r="J30" s="33" t="inlineStr">
         <is>
-          <t>k0CfyHTmb4Q</t>
+          <t>tO1C8ABnsTo</t>
         </is>
       </c>
       <c r="L30" s="33" t="inlineStr">
@@ -51045,7 +51045,7 @@
       </c>
       <c r="J32" s="33" t="inlineStr">
         <is>
-          <t>lP8LLIjCe6Q</t>
+          <t>vimeo:1124774457</t>
         </is>
       </c>
       <c r="L32" s="33" t="inlineStr">
@@ -51100,7 +51100,7 @@
       </c>
       <c r="J33" s="33" t="inlineStr">
         <is>
-          <t>Pb4SnxpJLyE</t>
+          <t>vimeo:958338280</t>
         </is>
       </c>
       <c r="L33" s="33" t="inlineStr">
@@ -51265,7 +51265,7 @@
       </c>
       <c r="J36" s="33" t="inlineStr">
         <is>
-          <t>W3q1PQGXaps</t>
+          <t>vimeo:1066110069</t>
         </is>
       </c>
       <c r="L36" s="33" t="inlineStr">
@@ -51375,7 +51375,7 @@
       </c>
       <c r="J38" s="33" t="inlineStr">
         <is>
-          <t>fHoU4Z4uuck</t>
+          <t>vimeo:1130513290</t>
         </is>
       </c>
       <c r="L38" s="33" t="inlineStr">
@@ -51485,7 +51485,7 @@
       </c>
       <c r="J40" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1074788616</t>
+          <t>vimeo:1074524233</t>
         </is>
       </c>
       <c r="L40" s="33" t="inlineStr">
@@ -51595,7 +51595,7 @@
       </c>
       <c r="J42" s="33" t="inlineStr">
         <is>
-          <t>QPJtgjoqtdw</t>
+          <t>uKT5bwMkOAw</t>
         </is>
       </c>
       <c r="K42" s="33" t="n"/>
@@ -51706,7 +51706,7 @@
       </c>
       <c r="J44" s="33" t="inlineStr">
         <is>
-          <t>pwLergHG81c</t>
+          <t>vimeo:1059963620</t>
         </is>
       </c>
       <c r="L44" s="33" t="inlineStr">
@@ -51761,7 +51761,7 @@
       </c>
       <c r="J45" s="33" t="inlineStr">
         <is>
-          <t>hlqerWZSCpE</t>
+          <t>vimeo:1023704952</t>
         </is>
       </c>
       <c r="L45" s="33" t="inlineStr">
@@ -51816,7 +51816,7 @@
       </c>
       <c r="J46" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1074788616</t>
+          <t>vimeo:1074524233</t>
         </is>
       </c>
       <c r="L46" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Final Updated Video Link (Large Batch 100+)
</commit_message>
<xml_diff>
--- a/Brain_Cannesdy_Brand_Experience_2025.xlsx
+++ b/Brain_Cannesdy_Brand_Experience_2025.xlsx
@@ -1829,7 +1829,7 @@
       </c>
       <c r="J15" s="33" t="inlineStr">
         <is>
-          <t>C5hcv9fi0VQ</t>
+          <t>mp4:videos/clandestination.mp4</t>
         </is>
       </c>
       <c r="L15" s="33" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="J18" s="33" t="inlineStr">
         <is>
-          <t>LDbcqtL9zP8</t>
+          <t>vimeo:1090130974</t>
         </is>
       </c>
       <c r="L18" s="33" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="J27" s="33" t="inlineStr">
         <is>
-          <t>zEQhgXoMsdY</t>
+          <t>vimeo:1153574180</t>
         </is>
       </c>
       <c r="L27" s="33" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J32" s="33" t="inlineStr">
         <is>
-          <t>Z_lbVlhO9HE</t>
+          <t>vimeo:1000498095</t>
         </is>
       </c>
       <c r="L32" s="33" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="J36" s="33" t="inlineStr">
         <is>
-          <t>z2T-Rh838GA</t>
+          <t>vimeo:1078276871</t>
         </is>
       </c>
       <c r="L36" s="33" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="J38" s="33" t="inlineStr">
         <is>
-          <t>uUDgTwzWz5U</t>
+          <t>Rz2FWiJq4Mw</t>
         </is>
       </c>
       <c r="L38" s="33" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="J40" s="33" t="inlineStr">
         <is>
-          <t>lqnGQri4ckE</t>
+          <t>vimeo:1086909960</t>
         </is>
       </c>
       <c r="L40" s="33" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="J46" s="33" t="inlineStr">
         <is>
-          <t>_GNOgJWpfK8</t>
+          <t>vimeo:1093963149</t>
         </is>
       </c>
       <c r="L46" s="33" t="inlineStr">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="J48" s="33" t="inlineStr">
         <is>
-          <t>9HpJtpvtrhs</t>
+          <t>vimeo:1149640616</t>
         </is>
       </c>
       <c r="L48" s="33" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="J58" s="33" t="inlineStr">
         <is>
-          <t>7kRgxEIhX38</t>
+          <t>vimeo:1083484983</t>
         </is>
       </c>
       <c r="L58" s="33" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="J59" s="33" t="inlineStr">
         <is>
-          <t>cjnTY_qX2wM</t>
+          <t>vimeo:1152835840</t>
         </is>
       </c>
       <c r="L59" s="33" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="J68" s="33" t="inlineStr">
         <is>
-          <t>2B2-joqRoHc</t>
+          <t>vimeo:1105993323</t>
         </is>
       </c>
       <c r="L68" s="33" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="J3" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1093399082</t>
+          <t>3ur8Gor_h-4</t>
         </is>
       </c>
       <c r="L3" s="33" t="inlineStr">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="J4" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094885092</t>
+          <t>vimeo:1094885092/740ca01ef6</t>
         </is>
       </c>
       <c r="L4" s="33" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="J7" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094791063</t>
+          <t>vimeo:1094791063/08d1ef48b6</t>
         </is>
       </c>
       <c r="L7" s="33" t="inlineStr">
@@ -6647,7 +6647,7 @@
       </c>
       <c r="J7" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1092193619</t>
+          <t>MnF0kip489Y</t>
         </is>
       </c>
       <c r="L7" s="33" t="inlineStr">
@@ -6698,6 +6698,11 @@
       <c r="I8" s="33" t="inlineStr">
         <is>
           <t>https://ascentialcdn.filespin.io/api/v1/conversion/9f8364b5c9b847aa83fb8ea7b62628d8</t>
+        </is>
+      </c>
+      <c r="J8" s="33" t="inlineStr">
+        <is>
+          <t>eAqaciBGz3k</t>
         </is>
       </c>
       <c r="L8" s="33" t="inlineStr">
@@ -6897,7 +6902,7 @@
       </c>
       <c r="J3" s="33" t="inlineStr">
         <is>
-          <t>0-vXeXH0PTg</t>
+          <t>vimeo:1097204731</t>
         </is>
       </c>
       <c r="L3" s="33" t="inlineStr">
@@ -7117,7 +7122,7 @@
       </c>
       <c r="J7" s="33" t="inlineStr">
         <is>
-          <t>8NxoqgLXy2E</t>
+          <t>vimeo:1186233105</t>
         </is>
       </c>
       <c r="L7" s="33" t="inlineStr">
@@ -7592,7 +7597,7 @@
       </c>
       <c r="J5" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094223404</t>
+          <t>5H6KsnFazXM</t>
         </is>
       </c>
       <c r="L5" s="33" t="inlineStr">
@@ -8452,7 +8457,7 @@
       </c>
       <c r="J8" s="33" t="inlineStr">
         <is>
-          <t>kfnhUWM876k</t>
+          <t>vimeo:1094309286</t>
         </is>
       </c>
       <c r="L8" s="33" t="inlineStr">
@@ -8617,7 +8622,7 @@
       </c>
       <c r="J11" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094885255</t>
+          <t>vimeo:1094885255/793d3aa7b3</t>
         </is>
       </c>
       <c r="L11" s="33" t="inlineStr">
@@ -8927,7 +8932,7 @@
       </c>
       <c r="J2" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094885157</t>
+          <t>vimeo:1096001831</t>
         </is>
       </c>
       <c r="L2" s="33" t="inlineStr">
@@ -9367,7 +9372,7 @@
       </c>
       <c r="J10" s="33" t="inlineStr">
         <is>
-          <t>kfnhUWM876k</t>
+          <t>vimeo:1094309286</t>
         </is>
       </c>
       <c r="L10" s="33" t="inlineStr">
@@ -9582,7 +9587,7 @@
       </c>
       <c r="J14" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1095117362</t>
+          <t>vimeo:1095117362/9d5a6fba02</t>
         </is>
       </c>
       <c r="L14" s="33" t="inlineStr">
@@ -9692,7 +9697,7 @@
       </c>
       <c r="J16" s="33" t="inlineStr">
         <is>
-          <t>vimeo:951451298</t>
+          <t>zBQtfBKPuYU</t>
         </is>
       </c>
       <c r="L16" s="33" t="inlineStr">
@@ -10373,7 +10378,7 @@
       </c>
       <c r="J11" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094223419</t>
+          <t>vimeo:1152941322</t>
         </is>
       </c>
       <c r="L11" s="33" t="inlineStr">
@@ -10428,7 +10433,7 @@
       </c>
       <c r="J12" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094221778</t>
+          <t>vimeo:1094221778/ad37613e9a</t>
         </is>
       </c>
       <c r="L12" s="33" t="inlineStr">
@@ -10959,7 +10964,7 @@
       </c>
       <c r="J4" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1003184179</t>
+          <t>pn80885I5OY</t>
         </is>
       </c>
       <c r="L4" s="33" t="inlineStr">
@@ -11749,7 +11754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="34" min="1" max="1"/>
@@ -12039,7 +12044,7 @@
       </c>
       <c r="J5" s="92" t="inlineStr">
         <is>
-          <t>gD1XqvQaMR0</t>
+          <t>sH5Jk7ywBLc</t>
         </is>
       </c>
       <c r="L5" s="33" t="inlineStr">
@@ -12149,7 +12154,7 @@
       </c>
       <c r="J7" s="92" t="inlineStr">
         <is>
-          <t>LDbcqtL9zP8</t>
+          <t>vimeo:1090130974</t>
         </is>
       </c>
       <c r="L7" s="33" t="inlineStr">
@@ -12204,7 +12209,7 @@
       </c>
       <c r="J8" s="92" t="inlineStr">
         <is>
-          <t>vimeo:1093833122</t>
+          <t>vimeo:1105218555</t>
         </is>
       </c>
       <c r="L8" s="33" t="inlineStr">
@@ -12229,14 +12234,14 @@
       </c>
       <c r="D9" s="92" t="inlineStr">
         <is>
+          <t>Coors Brewing Company</t>
+        </is>
+      </c>
+      <c r="E9" s="92" t="inlineStr">
+        <is>
           <t>Coors Light</t>
         </is>
       </c>
-      <c r="E9" s="92" t="inlineStr">
-        <is>
-          <t>Coors Light</t>
-        </is>
-      </c>
       <c r="F9" s="92" t="inlineStr">
         <is>
           <t>Alma Advertising Agency</t>
@@ -12259,7 +12264,7 @@
       </c>
       <c r="J9" s="92" t="inlineStr">
         <is>
-          <t>BqqqBYEADPg</t>
+          <t>vimeo:1086177966</t>
         </is>
       </c>
       <c r="L9" s="33" t="inlineStr">
@@ -12369,7 +12374,7 @@
       </c>
       <c r="J11" s="92" t="inlineStr">
         <is>
-          <t>gD1XqvQaMR0</t>
+          <t>sH5Jk7ywBLc</t>
         </is>
       </c>
       <c r="L11" s="33" t="inlineStr">
@@ -12424,7 +12429,7 @@
       </c>
       <c r="J12" s="92" t="inlineStr">
         <is>
-          <t>t10NTUNmF8c</t>
+          <t>vimeo:1081566541</t>
         </is>
       </c>
       <c r="L12" s="33" t="inlineStr">
@@ -12534,7 +12539,7 @@
       </c>
       <c r="J14" s="92" t="inlineStr">
         <is>
-          <t>cjnTY_qX2wM</t>
+          <t>UkdMtj9108s</t>
         </is>
       </c>
       <c r="L14" s="33" t="inlineStr">
@@ -12980,6 +12985,258 @@
       <c r="L22" s="33" t="inlineStr">
         <is>
           <t>https://www.lovethework.com/work/entries/sounds-right-759882</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="33" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>2. High Energy Boyfriend</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="inlineStr">
+        <is>
+          <t>Fusion Energy Drink</t>
+        </is>
+      </c>
+      <c r="F23" s="33" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H23" s="33" t="inlineStr">
+        <is>
+          <t>B03 - Script</t>
+        </is>
+      </c>
+      <c r="I23" s="33" t="inlineStr">
+        <is>
+          <t>https://ascentialcdn.filespin.io/api/v1/storyboard/846afe3e468240929823119e42cf3b99/storyboard_000008.jpg</t>
+        </is>
+      </c>
+      <c r="J23" s="33" t="inlineStr">
+        <is>
+          <t>vimeo:1105218613</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>3. High Energy Dad</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="inlineStr">
+        <is>
+          <t>Fusion Energy Drink</t>
+        </is>
+      </c>
+      <c r="F24" s="33" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H24" s="33" t="inlineStr">
+        <is>
+          <t>B03 - Script</t>
+        </is>
+      </c>
+      <c r="I24" s="33" t="inlineStr">
+        <is>
+          <t>https://ascentialcdn.filespin.io/api/v1/storyboard/846afe3e468240929823119e42cf3b99/storyboard_000008.jpg</t>
+        </is>
+      </c>
+      <c r="J24" s="33" t="inlineStr">
+        <is>
+          <t>vimeo:1105218658</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>Cold Detector</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>Coors Brewing Company</t>
+        </is>
+      </c>
+      <c r="F25" s="33" t="inlineStr">
+        <is>
+          <t>Alma Advertising Agency</t>
+        </is>
+      </c>
+      <c r="G25" s="33" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="H25" s="33" t="inlineStr">
+        <is>
+          <t>B04 - Casting &amp; Performance</t>
+        </is>
+      </c>
+      <c r="I25" s="33" t="inlineStr">
+        <is>
+          <t>digital-presentation-images/audio-and-radio-coors-light-chill-enough.webp</t>
+        </is>
+      </c>
+      <c r="J25" s="33" t="inlineStr">
+        <is>
+          <t>vimeo:1086178012</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>Mountain Cold</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>Coors Brewing Company</t>
+        </is>
+      </c>
+      <c r="F26" s="33" t="inlineStr">
+        <is>
+          <t>Alma Advertising Agency</t>
+        </is>
+      </c>
+      <c r="G26" s="33" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="H26" s="33" t="inlineStr">
+        <is>
+          <t>B04 - Casting &amp; Performance</t>
+        </is>
+      </c>
+      <c r="I26" s="33" t="inlineStr">
+        <is>
+          <t>digital-presentation-images/audio-and-radio-coors-light-chill-enough.webp</t>
+        </is>
+      </c>
+      <c r="J26" s="33" t="inlineStr">
+        <is>
+          <t>vimeo:1086178036</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="33" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="C27" s="33" t="inlineStr">
+        <is>
+          <t>Spill the Tea</t>
+        </is>
+      </c>
+      <c r="D27" s="33" t="inlineStr">
+        <is>
+          <t>Hansa Pilsener</t>
+        </is>
+      </c>
+      <c r="F27" s="33" t="inlineStr">
+        <is>
+          <t>Joe Public</t>
+        </is>
+      </c>
+      <c r="G27" s="33" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="H27" s="33" t="inlineStr">
+        <is>
+          <t>B03 - Script</t>
+        </is>
+      </c>
+      <c r="I27" s="33" t="inlineStr">
+        <is>
+          <t>https://ascentialcdn.filespin.io/api/v1/storyboard/0bca684772274dd9a6e2c0c6cd401876/storyboard_000008.jpg</t>
+        </is>
+      </c>
+      <c r="J27" s="33" t="inlineStr">
+        <is>
+          <t>vimeo:1032236549</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="C28" s="33" t="inlineStr">
+        <is>
+          <t>Okrrr</t>
+        </is>
+      </c>
+      <c r="D28" s="33" t="inlineStr">
+        <is>
+          <t>Hansa Pilsener</t>
+        </is>
+      </c>
+      <c r="F28" s="33" t="inlineStr">
+        <is>
+          <t>Joe Public</t>
+        </is>
+      </c>
+      <c r="G28" s="33" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="H28" s="33" t="inlineStr">
+        <is>
+          <t>B03 - Script</t>
+        </is>
+      </c>
+      <c r="I28" s="33" t="inlineStr">
+        <is>
+          <t>https://ascentialcdn.filespin.io/api/v1/storyboard/0bca684772274dd9a6e2c0c6cd401876/storyboard_000008.jpg</t>
+        </is>
+      </c>
+      <c r="J28" s="33" t="inlineStr">
+        <is>
+          <t>vimeo:1022471976</t>
         </is>
       </c>
     </row>
@@ -13329,7 +13586,7 @@
       </c>
       <c r="J6" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1092193619</t>
+          <t>MnF0kip489Y</t>
         </is>
       </c>
       <c r="L6" s="33" t="inlineStr">
@@ -13549,7 +13806,7 @@
       </c>
       <c r="J10" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094885157</t>
+          <t>vimeo:1096001831</t>
         </is>
       </c>
       <c r="L10" s="33" t="inlineStr">
@@ -14959,7 +15216,7 @@
       </c>
       <c r="J17" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094885234</t>
+          <t>vimeo:1095764716</t>
         </is>
       </c>
       <c r="L17" s="33" t="inlineStr">
@@ -15379,7 +15636,7 @@
       </c>
       <c r="J3" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094956645</t>
+          <t>-4o8bCc6-GM</t>
         </is>
       </c>
       <c r="L3" s="33" t="inlineStr">
@@ -15544,7 +15801,7 @@
       </c>
       <c r="J6" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1080276069</t>
+          <t>vimeo:1103262672</t>
         </is>
       </c>
       <c r="L6" s="33" t="inlineStr">
@@ -15654,7 +15911,7 @@
       </c>
       <c r="J8" s="33" t="inlineStr">
         <is>
-          <t>vimeo:943372451</t>
+          <t>0C3VQ6MwfIE</t>
         </is>
       </c>
       <c r="L8" s="33" t="inlineStr">
@@ -15874,7 +16131,7 @@
       </c>
       <c r="J12" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094956645</t>
+          <t>-4o8bCc6-GM</t>
         </is>
       </c>
       <c r="L12" s="33" t="inlineStr">
@@ -15929,7 +16186,7 @@
       </c>
       <c r="J13" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1093757553</t>
+          <t>t8o4ulxT1Cc</t>
         </is>
       </c>
       <c r="L13" s="33" t="inlineStr">
@@ -16039,7 +16296,7 @@
       </c>
       <c r="J15" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094223352</t>
+          <t>vimeo:1126059126</t>
         </is>
       </c>
       <c r="L15" s="33" t="inlineStr">
@@ -16679,7 +16936,7 @@
       </c>
       <c r="J3" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1093757553</t>
+          <t>t8o4ulxT1Cc</t>
         </is>
       </c>
       <c r="L3" s="33" t="inlineStr">
@@ -16734,7 +16991,7 @@
       </c>
       <c r="J4" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094224675</t>
+          <t>vimeo:1094224675/e914bbd69e</t>
         </is>
       </c>
       <c r="L4" s="33" t="inlineStr">
@@ -17944,7 +18201,7 @@
       </c>
       <c r="J26" s="33" t="inlineStr">
         <is>
-          <t>3BbpfDvl6f4</t>
+          <t>vimeo:1081509339</t>
         </is>
       </c>
       <c r="L26" s="33" t="inlineStr">
@@ -18529,7 +18786,7 @@
       </c>
       <c r="J9" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094885200</t>
+          <t>vimeo:1094885200/2225619ba7</t>
         </is>
       </c>
       <c r="L9" s="33" t="inlineStr">
@@ -18749,7 +19006,7 @@
       </c>
       <c r="J13" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094791063</t>
+          <t>vimeo:1094791063/08d1ef48b6</t>
         </is>
       </c>
       <c r="L13" s="33" t="inlineStr">
@@ -22400,7 +22657,7 @@
       </c>
       <c r="J17" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1092193619</t>
+          <t>MnF0kip489Y</t>
         </is>
       </c>
       <c r="L17" s="33" t="inlineStr">
@@ -23280,7 +23537,7 @@
       </c>
       <c r="J33" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1092193619</t>
+          <t>MnF0kip489Y</t>
         </is>
       </c>
       <c r="L33" s="33" t="inlineStr">
@@ -23810,7 +24067,7 @@
       </c>
       <c r="J8" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094573277</t>
+          <t>vimeo:1153574180</t>
         </is>
       </c>
       <c r="L8" s="33" t="inlineStr">
@@ -23865,7 +24122,7 @@
       </c>
       <c r="J9" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1091835567</t>
+          <t>7i2fC6qJR2o</t>
         </is>
       </c>
       <c r="L9" s="33" t="inlineStr">
@@ -24360,7 +24617,7 @@
       </c>
       <c r="J18" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1092193619</t>
+          <t>MnF0kip489Y</t>
         </is>
       </c>
       <c r="L18" s="33" t="inlineStr">
@@ -24525,7 +24782,7 @@
       </c>
       <c r="J21" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094956645</t>
+          <t>-4o8bCc6-GM</t>
         </is>
       </c>
       <c r="L21" s="33" t="inlineStr">
@@ -24745,7 +25002,7 @@
       </c>
       <c r="J25" s="33" t="inlineStr">
         <is>
-          <t>Zc-U6PM9ilE</t>
+          <t>vimeo:1000498095</t>
         </is>
       </c>
       <c r="L25" s="33" t="inlineStr">
@@ -25515,7 +25772,7 @@
       </c>
       <c r="J39" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094578684</t>
+          <t>Rz2FWiJq4Mw</t>
         </is>
       </c>
       <c r="L39" s="33" t="inlineStr">
@@ -26100,7 +26357,7 @@
       </c>
       <c r="J4" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1083687587</t>
+          <t>vimeo:1174772200</t>
         </is>
       </c>
       <c r="K4" s="33" t="inlineStr">
@@ -26160,7 +26417,7 @@
       </c>
       <c r="J5" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1083687587</t>
+          <t>vimeo:1174772200</t>
         </is>
       </c>
       <c r="K5" s="33" t="inlineStr">
@@ -26276,7 +26533,7 @@
       </c>
       <c r="J7" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1083687587</t>
+          <t>vimeo:1174772200</t>
         </is>
       </c>
       <c r="K7" s="33" t="inlineStr">
@@ -26336,7 +26593,7 @@
       </c>
       <c r="J8" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1083687587</t>
+          <t>vimeo:1174772200</t>
         </is>
       </c>
       <c r="K8" s="33" t="inlineStr">
@@ -26396,7 +26653,7 @@
       </c>
       <c r="J9" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1083687587</t>
+          <t>vimeo:1174772200</t>
         </is>
       </c>
       <c r="K9" s="33" t="inlineStr">
@@ -27446,7 +27703,7 @@
       </c>
       <c r="J27" s="33" t="inlineStr">
         <is>
-          <t>mp4:https://video.adsoftheworld.com/ibifauwq5kyl1e6ba8ooyoj4clnb.mp4</t>
+          <t>v4Gr9oKgZR8</t>
         </is>
       </c>
       <c r="K27" s="33" t="inlineStr">
@@ -27741,7 +27998,7 @@
       </c>
       <c r="J32" s="33" t="inlineStr">
         <is>
-          <t>mp4:https://video.adsoftheworld.com/ibifauwq5kyl1e6ba8ooyoj4clnb.mp4</t>
+          <t>v4Gr9oKgZR8</t>
         </is>
       </c>
       <c r="K32" s="33" t="inlineStr">
@@ -27861,7 +28118,7 @@
       </c>
       <c r="J34" s="33" t="inlineStr">
         <is>
-          <t>mp4:https://video.adsoftheworld.com/ibifauwq5kyl1e6ba8ooyoj4clnb.mp4</t>
+          <t>v4Gr9oKgZR8</t>
         </is>
       </c>
       <c r="K34" s="33" t="inlineStr">
@@ -28276,7 +28533,7 @@
       </c>
       <c r="J41" s="33" t="inlineStr">
         <is>
-          <t>mp4:https://video.adsoftheworld.com/ibifauwq5kyl1e6ba8ooyoj4clnb.mp4</t>
+          <t>v4Gr9oKgZR8</t>
         </is>
       </c>
       <c r="K41" s="33" t="inlineStr">
@@ -29207,7 +29464,7 @@
       </c>
       <c r="J10" s="33" t="inlineStr">
         <is>
-          <t>d-mtDQXtR6I</t>
+          <t>RpvlshoKIrE</t>
         </is>
       </c>
       <c r="K10" s="33" t="inlineStr">
@@ -29267,7 +29524,7 @@
       </c>
       <c r="J11" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094581252</t>
+          <t>vimeo:1094581252/8afcb39440</t>
         </is>
       </c>
       <c r="L11" s="33" t="inlineStr">
@@ -30202,7 +30459,7 @@
       </c>
       <c r="J28" s="33" t="inlineStr">
         <is>
-          <t>LO4wamMlCKQ</t>
+          <t>vimeo:1067749538</t>
         </is>
       </c>
       <c r="L28" s="33" t="inlineStr">
@@ -30367,7 +30624,7 @@
       </c>
       <c r="J31" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094581252</t>
+          <t>vimeo:1094581252/8afcb39440</t>
         </is>
       </c>
       <c r="L31" s="33" t="inlineStr">
@@ -30917,7 +31174,7 @@
       </c>
       <c r="J41" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1094578702</t>
+          <t>vimeo:1094578702/cba6cf513a</t>
         </is>
       </c>
       <c r="L41" s="33" t="inlineStr">
@@ -31082,7 +31339,7 @@
       </c>
       <c r="J44" s="33" t="inlineStr">
         <is>
-          <t>d-mtDQXtR6I</t>
+          <t>RpvlshoKIrE</t>
         </is>
       </c>
       <c r="K44" s="33" t="inlineStr">
@@ -36004,7 +36261,7 @@
       </c>
       <c r="J28" s="33" t="inlineStr">
         <is>
-          <t>d-mtDQXtR6I</t>
+          <t>RpvlshoKIrE</t>
         </is>
       </c>
       <c r="L28" s="33" t="inlineStr">
@@ -38274,7 +38531,7 @@
       </c>
       <c r="J3" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1092193263</t>
+          <t>vimeo:1109390480</t>
         </is>
       </c>
       <c r="L3" s="33" t="inlineStr">
@@ -38384,7 +38641,7 @@
       </c>
       <c r="J5" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1092193263</t>
+          <t>vimeo:1109390480</t>
         </is>
       </c>
       <c r="L5" s="33" t="inlineStr">
@@ -38494,7 +38751,7 @@
       </c>
       <c r="J7" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1092193263</t>
+          <t>vimeo:1109390480</t>
         </is>
       </c>
       <c r="L7" s="33" t="inlineStr">
@@ -39792,7 +40049,7 @@
       </c>
       <c r="J9" s="33" t="inlineStr">
         <is>
-          <t>GR2NjU6fhZw</t>
+          <t>vimeo:1167690695</t>
         </is>
       </c>
       <c r="K9" s="33" t="inlineStr">
@@ -39852,7 +40109,7 @@
       </c>
       <c r="J10" s="33" t="inlineStr">
         <is>
-          <t>9HpJtpvtrhs</t>
+          <t>vimeo:1167690695</t>
         </is>
       </c>
       <c r="K10" s="33" t="inlineStr">
@@ -39912,7 +40169,7 @@
       </c>
       <c r="J11" s="33" t="inlineStr">
         <is>
-          <t>keOaQm6RpBg</t>
+          <t>vimeo:1167690695</t>
         </is>
       </c>
       <c r="K11" s="33" t="inlineStr">
@@ -40027,7 +40284,7 @@
       </c>
       <c r="J13" s="33" t="inlineStr">
         <is>
-          <t>7kRgxEIhX38</t>
+          <t>vimeo:1083484983</t>
         </is>
       </c>
       <c r="K13" s="33" t="inlineStr">
@@ -41414,19 +41671,19 @@
       </c>
       <c r="C38" s="107" t="inlineStr">
         <is>
-          <t>Too Yumm to Cheer\!</t>
+          <t>Too Yumm to Cheer!</t>
         </is>
       </c>
       <c r="D38" s="33" t="inlineStr">
         <is>
+          <t>Too Yumm!</t>
+        </is>
+      </c>
+      <c r="E38" s="33" t="inlineStr">
+        <is>
           <t>Too Yumm\!</t>
         </is>
       </c>
-      <c r="E38" s="33" t="inlineStr">
-        <is>
-          <t>Too Yumm\!</t>
-        </is>
-      </c>
       <c r="F38" s="33" t="inlineStr">
         <is>
           <t>FCB Kinnect</t>
@@ -41449,7 +41706,7 @@
       </c>
       <c r="J38" s="33" t="inlineStr">
         <is>
-          <t>2Kf-xAN5WCI</t>
+          <t>vimeo:1098960207</t>
         </is>
       </c>
       <c r="L38" s="33" t="inlineStr">
@@ -41504,7 +41761,7 @@
       </c>
       <c r="J39" s="33" t="inlineStr">
         <is>
-          <t>AwhMuPdXnUE</t>
+          <t>ZUXcFSbQ8LA</t>
         </is>
       </c>
       <c r="L39" s="33" t="inlineStr">
@@ -41559,7 +41816,7 @@
       </c>
       <c r="J40" s="33" t="inlineStr">
         <is>
-          <t>4j2UkSs-cSo</t>
+          <t>uIR17EmDu7g</t>
         </is>
       </c>
       <c r="L40" s="33" t="inlineStr">
@@ -41835,7 +42092,7 @@
       </c>
       <c r="J45" s="33" t="inlineStr">
         <is>
-          <t>ELBlWKeEqQQ</t>
+          <t>vimeo:1083484983</t>
         </is>
       </c>
       <c r="K45" s="33" t="inlineStr">
@@ -41895,7 +42152,7 @@
       </c>
       <c r="J46" s="33" t="inlineStr">
         <is>
-          <t>VGa1imApfdg</t>
+          <t>vimeo:1083484983</t>
         </is>
       </c>
       <c r="K46" s="33" t="inlineStr">
@@ -41955,7 +42212,7 @@
       </c>
       <c r="J47" s="33" t="inlineStr">
         <is>
-          <t>WcQDr4HxPKU</t>
+          <t>vimeo:1083484983</t>
         </is>
       </c>
       <c r="K47" s="33" t="inlineStr">
@@ -42075,7 +42332,7 @@
       </c>
       <c r="J49" s="33" t="inlineStr">
         <is>
-          <t>pitw8c1AXpI</t>
+          <t>ViJvHO9BxvU</t>
         </is>
       </c>
       <c r="K49" s="33" t="inlineStr">
@@ -42135,7 +42392,7 @@
       </c>
       <c r="J50" s="33" t="inlineStr">
         <is>
-          <t>pitw8c1AXpI</t>
+          <t>ViJvHO9BxvU</t>
         </is>
       </c>
       <c r="K50" s="33" t="inlineStr">
@@ -42195,7 +42452,7 @@
       </c>
       <c r="J51" s="33" t="inlineStr">
         <is>
-          <t>wXx6z3mDnVc</t>
+          <t>cnAXR4lk6R0</t>
         </is>
       </c>
       <c r="K51" s="33" t="inlineStr">
@@ -42315,7 +42572,7 @@
       </c>
       <c r="J53" s="33" t="inlineStr">
         <is>
-          <t>7GVxwv6ZNfw</t>
+          <t>cnAXR4lk6R0</t>
         </is>
       </c>
       <c r="K53" s="33" t="inlineStr">
@@ -42543,7 +42800,7 @@
       </c>
       <c r="J57" s="33" t="inlineStr">
         <is>
-          <t>5xRoKPmsEDI</t>
+          <t>W29029BIbvY</t>
         </is>
       </c>
       <c r="K57" s="33" t="inlineStr">
@@ -42603,7 +42860,7 @@
       </c>
       <c r="J58" s="33" t="inlineStr">
         <is>
-          <t>H6qzUSoN2Pc</t>
+          <t>W29029BIbvY</t>
         </is>
       </c>
       <c r="K58" s="33" t="inlineStr">
@@ -42663,7 +42920,7 @@
       </c>
       <c r="J59" s="33" t="inlineStr">
         <is>
-          <t>SDME83-pHnQ</t>
+          <t>W29029BIbvY</t>
         </is>
       </c>
       <c r="K59" s="33" t="inlineStr">
@@ -42943,7 +43200,7 @@
       </c>
       <c r="J64" s="33" t="inlineStr">
         <is>
-          <t>VGa1imApfdg</t>
+          <t>vimeo:1105993323</t>
         </is>
       </c>
       <c r="L64" s="33" t="inlineStr">
@@ -43383,7 +43640,7 @@
       </c>
       <c r="J72" s="33" t="inlineStr">
         <is>
-          <t>A8syQeFtBKc</t>
+          <t>vimeo:1083528511</t>
         </is>
       </c>
       <c r="L72" s="33" t="inlineStr">
@@ -43548,7 +43805,7 @@
       </c>
       <c r="J75" s="33" t="inlineStr">
         <is>
-          <t>pSNhG9OHuJw</t>
+          <t>vimeo:1073667667</t>
         </is>
       </c>
       <c r="L75" s="33" t="inlineStr">
@@ -43603,7 +43860,7 @@
       </c>
       <c r="J76" s="33" t="inlineStr">
         <is>
-          <t>8urf8-B-xrE</t>
+          <t>vimeo:1037597208</t>
         </is>
       </c>
       <c r="L76" s="33" t="inlineStr">
@@ -43913,7 +44170,7 @@
       </c>
       <c r="J3" s="80" t="inlineStr">
         <is>
-          <t>OzScknoWq6U</t>
+          <t>vimeo:1093371918</t>
         </is>
       </c>
       <c r="L3" s="33" t="inlineStr">
@@ -44078,7 +44335,7 @@
       </c>
       <c r="J6" s="80" t="inlineStr">
         <is>
-          <t>Z_lbVlhO9HE</t>
+          <t>vimeo:1000498095</t>
         </is>
       </c>
       <c r="L6" s="33" t="inlineStr">
@@ -44133,7 +44390,7 @@
       </c>
       <c r="J7" s="80" t="inlineStr">
         <is>
-          <t>Z_lbVlhO9HE</t>
+          <t>vimeo:1000498095</t>
         </is>
       </c>
       <c r="L7" s="33" t="inlineStr">
@@ -44463,7 +44720,7 @@
       </c>
       <c r="J13" s="80" t="inlineStr">
         <is>
-          <t>grgsxQjK0B4</t>
+          <t>vimeo:1093399093</t>
         </is>
       </c>
       <c r="L13" s="33" t="inlineStr">
@@ -44573,7 +44830,7 @@
       </c>
       <c r="J15" s="80" t="inlineStr">
         <is>
-          <t>vimeo:1094224721</t>
+          <t>vimeo:1117425129</t>
         </is>
       </c>
       <c r="L15" s="33" t="inlineStr">
@@ -44628,7 +44885,7 @@
       </c>
       <c r="J16" s="80" t="inlineStr">
         <is>
-          <t>7GVxwv6ZNfw</t>
+          <t>vimeo:1172671869</t>
         </is>
       </c>
       <c r="L16" s="33" t="inlineStr">
@@ -44793,7 +45050,7 @@
       </c>
       <c r="J19" s="80" t="inlineStr">
         <is>
-          <t>tmIsp44QoIA</t>
+          <t>vimeo:1015306334</t>
         </is>
       </c>
       <c r="L19" s="33" t="inlineStr">
@@ -45123,7 +45380,7 @@
       </c>
       <c r="J25" s="80" t="inlineStr">
         <is>
-          <t>I0W4kYosSXU</t>
+          <t>vimeo:1046618979</t>
         </is>
       </c>
       <c r="L25" s="33" t="inlineStr">
@@ -45178,7 +45435,7 @@
       </c>
       <c r="J26" s="80" t="inlineStr">
         <is>
-          <t>_GNOgJWpfK8</t>
+          <t>vimeo:1093963149</t>
         </is>
       </c>
       <c r="L26" s="33" t="inlineStr">
@@ -45288,7 +45545,7 @@
       </c>
       <c r="J28" s="80" t="inlineStr">
         <is>
-          <t>vimeo:1094221760</t>
+          <t>mp4:videos/workwear-for-kids.mp4</t>
         </is>
       </c>
       <c r="L28" s="33" t="inlineStr">
@@ -45343,7 +45600,7 @@
       </c>
       <c r="J29" s="80" t="inlineStr">
         <is>
-          <t>SqqroFfqKRc</t>
+          <t>U-twTRUItjY</t>
         </is>
       </c>
       <c r="L29" s="33" t="inlineStr">
@@ -45508,7 +45765,7 @@
       </c>
       <c r="J32" s="80" t="inlineStr">
         <is>
-          <t>grgsxQjK0B4</t>
+          <t>vimeo:1093399093</t>
         </is>
       </c>
       <c r="L32" s="33" t="inlineStr">
@@ -46425,7 +46682,7 @@
       </c>
       <c r="J16" s="80" t="inlineStr">
         <is>
-          <t>NZRnLh1U5HM</t>
+          <t>vimeo:1120973708</t>
         </is>
       </c>
       <c r="L16" s="33" t="inlineStr">
@@ -47580,7 +47837,7 @@
       </c>
       <c r="J37" s="80" t="inlineStr">
         <is>
-          <t>pixKU-we6XQ</t>
+          <t>vimeo:1077750867</t>
         </is>
       </c>
       <c r="L37" s="33" t="inlineStr">
@@ -47635,7 +47892,7 @@
       </c>
       <c r="J38" s="80" t="inlineStr">
         <is>
-          <t>_GNOgJWpfK8</t>
+          <t>vimeo:1093963149</t>
         </is>
       </c>
       <c r="L38" s="33" t="inlineStr">
@@ -47745,7 +48002,7 @@
       </c>
       <c r="J40" s="80" t="inlineStr">
         <is>
-          <t>mSPou5OfPyw</t>
+          <t>hLdCk8nEFcg</t>
         </is>
       </c>
       <c r="L40" s="33" t="inlineStr">
@@ -47910,7 +48167,7 @@
       </c>
       <c r="J43" s="80" t="inlineStr">
         <is>
-          <t>l3Sxq8LCXZA</t>
+          <t>2t2ysywk3do</t>
         </is>
       </c>
       <c r="L43" s="33" t="inlineStr">
@@ -47965,7 +48222,7 @@
       </c>
       <c r="J44" s="80" t="inlineStr">
         <is>
-          <t>GR2NjU6fhZw</t>
+          <t>vimeo:1094886574/76a7dd4cff</t>
         </is>
       </c>
       <c r="L44" s="33" t="inlineStr">
@@ -48130,7 +48387,7 @@
       </c>
       <c r="J47" s="80" t="inlineStr">
         <is>
-          <t>-xr4MO8lAjo</t>
+          <t>Rz2FWiJq4Mw</t>
         </is>
       </c>
       <c r="L47" s="33" t="inlineStr">
@@ -48295,7 +48552,7 @@
       </c>
       <c r="J50" s="80" t="inlineStr">
         <is>
-          <t>uUDgTwzWz5U</t>
+          <t>Rz2FWiJq4Mw</t>
         </is>
       </c>
       <c r="L50" s="33" t="inlineStr">
@@ -49065,7 +49322,7 @@
       </c>
       <c r="J64" s="80" t="inlineStr">
         <is>
-          <t>z2T-Rh838GA</t>
+          <t>vimeo:1078276871</t>
         </is>
       </c>
       <c r="L64" s="33" t="inlineStr">
@@ -49175,7 +49432,7 @@
       </c>
       <c r="J66" s="80" t="inlineStr">
         <is>
-          <t>A8syQeFtBKc</t>
+          <t>uv26WgWSh8g</t>
         </is>
       </c>
       <c r="L66" s="33" t="inlineStr">
@@ -51045,7 +51302,7 @@
       </c>
       <c r="J32" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1124774457</t>
+          <t>lP8LLIjCe6Q</t>
         </is>
       </c>
       <c r="L32" s="33" t="inlineStr">

</xml_diff>

<commit_message>
New fix for vimeo-hash videos.
</commit_message>
<xml_diff>
--- a/Brain_Cannesdy_Brand_Experience_2025.xlsx
+++ b/Brain_Cannesdy_Brand_Experience_2025.xlsx
@@ -26137,7 +26137,7 @@
       </c>
       <c r="J11" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1107064614</t>
+          <t>mp4:videos/naga-saint-eye-test.mp4</t>
         </is>
       </c>
       <c r="L11" s="33" t="inlineStr">
@@ -37205,7 +37205,7 @@
       </c>
       <c r="J51" s="33" t="inlineStr">
         <is>
-          <t>vimeo:1084518468</t>
+          <t>mp4:videos/bassi-vs-mens-facewash.mp4</t>
         </is>
       </c>
       <c r="L51" s="33" t="inlineStr">

</xml_diff>